<commit_message>
as_table_spec(): a plan written as code, back to a workbook
For turning an existing report into the template for a new study.  Read
from what the plan resolves to: roles, levels, labels, templates with
digits, layout, widths by name (.values), and the column header -- with
literals that are a column's key value turned back into {col}/{col1},
repeated cells into span = each and arm spanners into span = <key>, even
from a one-arm study.  What a sheet cannot say is listed, and the
workbook is run back through rtf_plan(spec = ) to report same pages.

The definition functions are renamed for what they define: table_spec(),
read_table_spec(), write_table_spec(), table_spec_template().  An
unnamed row key next to a constant heading keeps its own name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/ard-spec-local/study_localdata_v2.xlsx
+++ b/data-raw/ard-spec-local/study_localdata_v2.xlsx
@@ -393,7 +393,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rtfreporter の ARD 定義ファイル（spec_version 1）。rtf_plan(data; spec = read_ard_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
+          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。rtf_plan(data; spec = read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。rtf_plan(data; spec = read_ard_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
+          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。rtf_plan(data; spec = read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Report definition: read_report_spec(), rtf_report(), report_path()
Six sheets around the table, under the same output_id rule: report,
page, and the line sheets header / footer / titles / footnotes, keyed by
line -- the study's running header written once as default lines 1-2,
each report's titles on its own lines 3.., one default run-information
line 99 in the footer.  study gains output_path and program_dir.
rtf_report(spec, plan) builds the rtf_document carrying its program;
report_path() says where it goes.

A definition may span workbooks (a report workbook and content
workbooks): empty sheets and study keys may repeat, a sheet with rows
in two is refused.  A reader without output_id returns the whole study.

Sample report.xlsx beside study.xlsx; each report gives the identical
RTF to the document written as code.  data-raw/ard-spec-local carries
the user's report_localdata.xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/ard-spec-local/study_localdata_v2.xlsx
+++ b/data-raw/ard-spec-local/study_localdata_v2.xlsx
@@ -16,7 +16,13 @@
     <sheet name="columns" sheetId="7" r:id="rId7"/>
     <sheet name="style" sheetId="8" r:id="rId8"/>
     <sheet name="col_header" sheetId="9" r:id="rId9"/>
-    <sheet name="about" sheetId="10" r:id="rId10"/>
+    <sheet name="report" sheetId="10" r:id="rId10"/>
+    <sheet name="page" sheetId="11" r:id="rId11"/>
+    <sheet name="header" sheetId="12" r:id="rId12"/>
+    <sheet name="footer" sheetId="13" r:id="rId13"/>
+    <sheet name="titles" sheetId="14" r:id="rId14"/>
+    <sheet name="footnotes" sheetId="15" r:id="rId15"/>
+    <sheet name="about" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -360,7 +366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1415,34 +1421,170 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>about</t>
+          <t>(帳票全体)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>（読み方）</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>spec_version = 1</t>
+          <t>以下は表の周りの定義。read_report_spec(c(report.xlsx; tables.xlsx); output_id = ) で 1 冊でも分冊でも読める。同じシートに行があるのは 1 冊だけにする（空のシートと study は重なってよい）。rtf_report(spec; plan) で rtf_document、report_path(spec) で出力先。</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>output_path / program_dir</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>出力先フォルダ / プログラムのフォルダ（{PROGRAM} に使う）。</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>../tables / C:\study\tfl</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1 行 = 1 帳票（空欄 = 試験の既定）。type（table / listing / figure）、file（既定 {output_id}.rtf）、program（既定 {output_id}）、auto_section、section_align、auto_title、title_align、table_font_size / title_font_size / footnote_font_size（半ポイント）、page_header / page_footer（FALSE でその帳票だけ付けない）。</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>auto_section = TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1 行 = 1 帳票（空欄 = 試験の既定）。paper_size、orientation、width_in、height_in、margin_*_in、header_dist_in、footer_dist_in、font_size_half_points、title_format、footnote_format、title_width、footnote_width、markup。</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>A4 / landscape / 0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ページヘッダーの 1 行 = 1 行。line がキー：試験共通を空欄 output_id の 1・2 行目に、帳票のタイトルをその帳票の 3 行目以降に。left / center / right。文字のない行は空行。</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>1 / TAKEDA / / Interim Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>footer</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ページフッターの 1 行 = 1 行。帳票の脚注を 1 行目から、実行情報を空欄 output_id の 99 行目に 1 回だけ書けば全帳票の最後に付く。</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>99 / {PROGRAM}       Generated on: {DATETIME}</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>titles / footnotes</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>本文（表の上 / 下）のタイトル・脚注。書き方は header と同じ。</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1 / CV = Coefficient of variation</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>（差し込み記号）</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>{PAGE} {TOTAL_PAGES} {AUTO_PAGE} {AUTO_TOTAL_PAGES}（ページ番号）、{PROGRAM} {PROGRAM_NAME} {PROGRAM_DIR}（プログラム）、{DATETIME} {DATETIME:%Y-%m-%d}（作成日時）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>about</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>spec_version = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>(予約)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>次の版で読む予定のシート名。今は置いても読まれず、その旨のメッセージが出る。</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>titles / footnotes / page / header / footer / cell_styles</t>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>cell_styles / listing / listing_cols / figures</t>
         </is>
       </c>
     </row>
@@ -1453,6 +1595,328 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>program</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>auto_section</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>section_align</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>auto_title</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>title_align</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>table_font_size</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>title_font_size</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>footnote_font_size</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>page_header</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>page_footer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>paper_size</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>orientation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>width_in</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>height_in</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>margin_top_in</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>margin_bottom_in</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>margin_left_in</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>margin_right_in</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>header_dist_in</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>footer_dist_in</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>font_size_half_points</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>title_format</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>footnote_format</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>title_width</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>footnote_width</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>markup</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -1487,7 +1951,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1506,6 +1970,20 @@
       <c r="A2" t="inlineStr">
         <is>
           <t>rounding</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>output_path</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>program_dir</t>
         </is>
       </c>
     </row>

</xml_diff>